<commit_message>
dieu chinh PhoiNhapKho lan2
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/BM_TongHopGiaoNhanPhoiNhapKhoPKH.xlsx
+++ b/dataproduct.api/wwwroot/templates/BM_TongHopGiaoNhanPhoiNhapKhoPKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\03. ThongKePKH\DATAPRODUCT_V2\dataproduct.api\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B262C4-D3B7-4582-832D-252CA59A3FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8305F33E-3624-4782-AF23-7EF630ACF577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{77908C05-ABC3-4C3F-A6F5-1B05425144FB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="29">
   <si>
     <t>STT</t>
   </si>
@@ -96,13 +96,22 @@
     <t>Máy Đúc</t>
   </si>
   <si>
-    <t>PM giao nhận</t>
-  </si>
-  <si>
     <t>BK Mis</t>
   </si>
   <si>
-    <t>Chênh lệch</t>
+    <t>Tình trạng P.KH</t>
+  </si>
+  <si>
+    <t>Tình trạng QLCL</t>
+  </si>
+  <si>
+    <t>Tình trạng HRC</t>
+  </si>
+  <si>
+    <t>Nhập kho lần 1</t>
+  </si>
+  <si>
+    <t>Nhập kho lần 2</t>
   </si>
 </sst>
 </file>
@@ -393,6 +402,79 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -425,79 +507,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -859,7 +868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43BAB014-E6DF-4BFD-BF20-A00AB0E3B9F2}">
-  <dimension ref="A1:AU31"/>
+  <dimension ref="A1:AY31"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="1" customWidth="1"/>
@@ -881,287 +890,307 @@
     <col min="18" max="21" width="16.85546875" style="1" customWidth="1"/>
     <col min="22" max="22" width="33" style="1" customWidth="1"/>
     <col min="23" max="23" width="40.5703125" style="1" customWidth="1"/>
-    <col min="24" max="47" width="15" style="1" customWidth="1"/>
-    <col min="48" max="16384" width="9.140625" style="1"/>
+    <col min="24" max="51" width="15" style="1" customWidth="1"/>
+    <col min="52" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14"/>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+    <row r="1" spans="1:51" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="39"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
       <c r="E1" s="12"/>
     </row>
-    <row r="2" spans="1:47" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
+    <row r="2" spans="1:51" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
       <c r="E2" s="12"/>
     </row>
-    <row r="3" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15"/>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+      <c r="S3" s="40"/>
+      <c r="T3" s="40"/>
+      <c r="U3" s="40"/>
     </row>
-    <row r="4" spans="1:47" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:51" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41"/>
+      <c r="P4" s="41"/>
+      <c r="Q4" s="41"/>
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="41"/>
     </row>
-    <row r="5" spans="1:47" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:51" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
-      <c r="I5" s="46" t="s">
+      <c r="I5" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="46"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="46"/>
-      <c r="M5" s="46"/>
-      <c r="N5" s="46"/>
-      <c r="O5" s="46"/>
-      <c r="P5" s="46"/>
-      <c r="Q5" s="46"/>
-      <c r="R5" s="46"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="46"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="46"/>
-      <c r="X5" s="47" t="s">
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y5" s="19"/>
+      <c r="Z5" s="19"/>
+      <c r="AA5" s="19"/>
+      <c r="AB5" s="19"/>
+      <c r="AC5" s="19"/>
+      <c r="AD5" s="19"/>
+      <c r="AE5" s="19"/>
+      <c r="AF5" s="19"/>
+      <c r="AG5" s="19"/>
+      <c r="AH5" s="19"/>
+      <c r="AI5" s="19"/>
+      <c r="AJ5" s="19"/>
+      <c r="AK5" s="19"/>
+      <c r="AL5" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="AM5" s="20"/>
+      <c r="AN5" s="20"/>
+      <c r="AO5" s="20"/>
+      <c r="AP5" s="20"/>
+      <c r="AQ5" s="20"/>
+      <c r="AR5" s="20"/>
+      <c r="AS5" s="20"/>
+      <c r="AT5" s="20"/>
+      <c r="AU5" s="20"/>
+      <c r="AV5" s="20"/>
+      <c r="AW5" s="20"/>
+      <c r="AX5" s="20"/>
+      <c r="AY5" s="20"/>
+    </row>
+    <row r="6" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="14"/>
+      <c r="K6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="23"/>
+      <c r="M6" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="27"/>
+      <c r="O6" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="30"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="S6" s="14"/>
+      <c r="T6" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="U6" s="35" t="s">
+        <v>4</v>
+      </c>
+      <c r="V6" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="W6" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="X6" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="AA6" s="23"/>
+      <c r="AB6" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC6" s="27"/>
+      <c r="AD6" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE6" s="30"/>
+      <c r="AF6" s="27"/>
+      <c r="AG6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH6" s="14"/>
+      <c r="AI6" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="AJ6" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="AK6" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="Y5" s="47"/>
-      <c r="Z5" s="47"/>
-      <c r="AA5" s="47"/>
-      <c r="AB5" s="47"/>
-      <c r="AC5" s="47"/>
-      <c r="AD5" s="47"/>
-      <c r="AE5" s="47"/>
-      <c r="AF5" s="47"/>
-      <c r="AG5" s="47"/>
-      <c r="AH5" s="47"/>
-      <c r="AI5" s="47"/>
-      <c r="AJ5" s="48" t="s">
+      <c r="AL6" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="AM6" s="14"/>
+      <c r="AN6" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="AO6" s="23"/>
+      <c r="AP6" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="AQ6" s="27"/>
+      <c r="AR6" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="AS6" s="30"/>
+      <c r="AT6" s="27"/>
+      <c r="AU6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="AV6" s="14"/>
+      <c r="AW6" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="AX6" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="AK5" s="48"/>
-      <c r="AL5" s="48"/>
-      <c r="AM5" s="48"/>
-      <c r="AN5" s="48"/>
-      <c r="AO5" s="48"/>
-      <c r="AP5" s="48"/>
-      <c r="AQ5" s="48"/>
-      <c r="AR5" s="48"/>
-      <c r="AS5" s="48"/>
-      <c r="AT5" s="48"/>
-      <c r="AU5" s="48"/>
+      <c r="AY6" s="15" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="6" spans="1:47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="H6" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="J6" s="30"/>
-      <c r="K6" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="33"/>
-      <c r="M6" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="N6" s="37"/>
-      <c r="O6" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="P6" s="40"/>
-      <c r="Q6" s="37"/>
-      <c r="R6" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="S6" s="30"/>
-      <c r="T6" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="U6" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="V6" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="W6" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="X6" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="Y6" s="30"/>
-      <c r="Z6" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC6" s="37"/>
-      <c r="AD6" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="AE6" s="40"/>
-      <c r="AF6" s="37"/>
-      <c r="AG6" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="AH6" s="30"/>
-      <c r="AI6" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ6" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="AK6" s="30"/>
-      <c r="AL6" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM6" s="33"/>
-      <c r="AN6" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="AO6" s="37"/>
-      <c r="AP6" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="AQ6" s="40"/>
-      <c r="AR6" s="37"/>
-      <c r="AS6" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="AT6" s="30"/>
-      <c r="AU6" s="42" t="s">
-        <v>20</v>
-      </c>
+    <row r="7" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="42"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="25"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="29"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="31"/>
+      <c r="Q7" s="29"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="36"/>
+      <c r="V7" s="36"/>
+      <c r="W7" s="33"/>
+      <c r="X7" s="21"/>
+      <c r="Y7" s="21"/>
+      <c r="Z7" s="24"/>
+      <c r="AA7" s="25"/>
+      <c r="AB7" s="28"/>
+      <c r="AC7" s="29"/>
+      <c r="AD7" s="28"/>
+      <c r="AE7" s="31"/>
+      <c r="AF7" s="29"/>
+      <c r="AG7" s="14"/>
+      <c r="AH7" s="14"/>
+      <c r="AI7" s="16"/>
+      <c r="AJ7" s="16"/>
+      <c r="AK7" s="16"/>
+      <c r="AL7" s="21"/>
+      <c r="AM7" s="21"/>
+      <c r="AN7" s="24"/>
+      <c r="AO7" s="25"/>
+      <c r="AP7" s="28"/>
+      <c r="AQ7" s="29"/>
+      <c r="AR7" s="28"/>
+      <c r="AS7" s="31"/>
+      <c r="AT7" s="29"/>
+      <c r="AU7" s="14"/>
+      <c r="AV7" s="14"/>
+      <c r="AW7" s="16"/>
+      <c r="AX7" s="16"/>
+      <c r="AY7" s="16"/>
     </row>
-    <row r="7" spans="1:47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="38"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="38"/>
-      <c r="P7" s="41"/>
-      <c r="Q7" s="39"/>
-      <c r="R7" s="30"/>
-      <c r="S7" s="30"/>
-      <c r="T7" s="43"/>
-      <c r="U7" s="28"/>
-      <c r="V7" s="28"/>
-      <c r="W7" s="25"/>
-      <c r="X7" s="31"/>
-      <c r="Y7" s="31"/>
-      <c r="Z7" s="34"/>
-      <c r="AA7" s="35"/>
-      <c r="AB7" s="38"/>
-      <c r="AC7" s="39"/>
-      <c r="AD7" s="38"/>
-      <c r="AE7" s="41"/>
-      <c r="AF7" s="39"/>
-      <c r="AG7" s="30"/>
-      <c r="AH7" s="30"/>
-      <c r="AI7" s="43"/>
-      <c r="AJ7" s="31"/>
-      <c r="AK7" s="31"/>
-      <c r="AL7" s="34"/>
-      <c r="AM7" s="35"/>
-      <c r="AN7" s="38"/>
-      <c r="AO7" s="39"/>
-      <c r="AP7" s="38"/>
-      <c r="AQ7" s="41"/>
-      <c r="AR7" s="39"/>
-      <c r="AS7" s="30"/>
-      <c r="AT7" s="30"/>
-      <c r="AU7" s="43"/>
-    </row>
-    <row r="8" spans="1:47" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="20"/>
+    <row r="8" spans="1:51" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="42"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="45"/>
       <c r="I8" s="5" t="s">
         <v>12</v>
       </c>
@@ -1195,10 +1224,10 @@
       <c r="S8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="T8" s="44"/>
-      <c r="U8" s="29"/>
-      <c r="V8" s="29"/>
-      <c r="W8" s="26"/>
+      <c r="T8" s="17"/>
+      <c r="U8" s="37"/>
+      <c r="V8" s="37"/>
+      <c r="W8" s="34"/>
       <c r="X8" s="5" t="s">
         <v>12</v>
       </c>
@@ -1232,14 +1261,10 @@
       <c r="AH8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="AI8" s="44"/>
-      <c r="AJ8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="AK8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="AL8" s="3" t="s">
+      <c r="AI8" s="17"/>
+      <c r="AJ8" s="17"/>
+      <c r="AK8" s="17"/>
+      <c r="AL8" s="5" t="s">
         <v>12</v>
       </c>
       <c r="AM8" s="11" t="s">
@@ -1254,21 +1279,29 @@
       <c r="AP8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="AQ8" s="3" t="s">
+      <c r="AQ8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="AR8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AS8" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="AR8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="AS8" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="AT8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="AU8" s="44"/>
+      <c r="AU8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AV8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="AW8" s="17"/>
+      <c r="AX8" s="17"/>
+      <c r="AY8" s="17"/>
     </row>
-    <row r="9" spans="1:47" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:51" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
       <c r="B9" s="7"/>
       <c r="C9" s="8"/>
@@ -1294,38 +1327,42 @@
       </c>
       <c r="V9" s="9"/>
       <c r="W9" s="10"/>
-      <c r="X9" s="45"/>
-      <c r="Y9" s="45"/>
-      <c r="Z9" s="45"/>
-      <c r="AA9" s="45"/>
-      <c r="AB9" s="45"/>
-      <c r="AC9" s="45"/>
-      <c r="AD9" s="45"/>
-      <c r="AE9" s="45"/>
-      <c r="AF9" s="45"/>
-      <c r="AG9" s="45"/>
-      <c r="AH9" s="45"/>
-      <c r="AI9" s="45"/>
-      <c r="AJ9" s="45"/>
-      <c r="AK9" s="45"/>
-      <c r="AL9" s="45"/>
-      <c r="AM9" s="45"/>
-      <c r="AN9" s="45"/>
-      <c r="AO9" s="45"/>
-      <c r="AP9" s="45"/>
-      <c r="AQ9" s="45"/>
-      <c r="AR9" s="45"/>
-      <c r="AS9" s="45"/>
-      <c r="AT9" s="45"/>
-      <c r="AU9" s="45"/>
+      <c r="X9" s="13"/>
+      <c r="Y9" s="13"/>
+      <c r="Z9" s="13"/>
+      <c r="AA9" s="13"/>
+      <c r="AB9" s="13"/>
+      <c r="AC9" s="13"/>
+      <c r="AD9" s="13"/>
+      <c r="AE9" s="13"/>
+      <c r="AF9" s="13"/>
+      <c r="AG9" s="13"/>
+      <c r="AH9" s="13"/>
+      <c r="AI9" s="13"/>
+      <c r="AJ9" s="13"/>
+      <c r="AK9" s="13"/>
+      <c r="AL9" s="13"/>
+      <c r="AM9" s="13"/>
+      <c r="AN9" s="13"/>
+      <c r="AO9" s="13"/>
+      <c r="AP9" s="13"/>
+      <c r="AQ9" s="13"/>
+      <c r="AR9" s="13"/>
+      <c r="AS9" s="13"/>
+      <c r="AT9" s="13"/>
+      <c r="AU9" s="13"/>
+      <c r="AV9" s="13"/>
+      <c r="AW9" s="13"/>
+      <c r="AX9" s="13"/>
+      <c r="AY9" s="13"/>
     </row>
-    <row r="10" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:47" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:51" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1342,31 +1379,11 @@
     <row r="30" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="AS6:AT7"/>
-    <mergeCell ref="AU6:AU8"/>
-    <mergeCell ref="I5:W5"/>
-    <mergeCell ref="X5:AI5"/>
-    <mergeCell ref="AJ5:AU5"/>
+  <mergeCells count="39">
+    <mergeCell ref="AJ6:AJ8"/>
     <mergeCell ref="AI6:AI8"/>
-    <mergeCell ref="AJ6:AK7"/>
-    <mergeCell ref="AL6:AM7"/>
-    <mergeCell ref="AN6:AO7"/>
-    <mergeCell ref="AP6:AR7"/>
-    <mergeCell ref="X6:Y7"/>
-    <mergeCell ref="Z6:AA7"/>
-    <mergeCell ref="AB6:AC7"/>
-    <mergeCell ref="AD6:AF7"/>
-    <mergeCell ref="AG6:AH7"/>
-    <mergeCell ref="W6:W8"/>
-    <mergeCell ref="V6:V8"/>
-    <mergeCell ref="U6:U8"/>
-    <mergeCell ref="I6:J7"/>
-    <mergeCell ref="R6:S7"/>
-    <mergeCell ref="K6:L7"/>
-    <mergeCell ref="M6:N7"/>
-    <mergeCell ref="O6:Q7"/>
-    <mergeCell ref="T6:T8"/>
+    <mergeCell ref="AX6:AX8"/>
+    <mergeCell ref="AW6:AW8"/>
     <mergeCell ref="G6:G8"/>
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="A3:U3"/>
@@ -1378,6 +1395,30 @@
     <mergeCell ref="F6:F8"/>
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="E6:E8"/>
+    <mergeCell ref="V6:V8"/>
+    <mergeCell ref="U6:U8"/>
+    <mergeCell ref="I6:J7"/>
+    <mergeCell ref="R6:S7"/>
+    <mergeCell ref="K6:L7"/>
+    <mergeCell ref="M6:N7"/>
+    <mergeCell ref="O6:Q7"/>
+    <mergeCell ref="T6:T8"/>
+    <mergeCell ref="AU6:AV7"/>
+    <mergeCell ref="AY6:AY8"/>
+    <mergeCell ref="I5:W5"/>
+    <mergeCell ref="X5:AK5"/>
+    <mergeCell ref="AL5:AY5"/>
+    <mergeCell ref="AK6:AK8"/>
+    <mergeCell ref="AL6:AM7"/>
+    <mergeCell ref="AN6:AO7"/>
+    <mergeCell ref="AP6:AQ7"/>
+    <mergeCell ref="AR6:AT7"/>
+    <mergeCell ref="X6:Y7"/>
+    <mergeCell ref="Z6:AA7"/>
+    <mergeCell ref="AB6:AC7"/>
+    <mergeCell ref="AD6:AF7"/>
+    <mergeCell ref="AG6:AH7"/>
+    <mergeCell ref="W6:W8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1561,20 +1602,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="7bdf782f-2886-4011-99ee-a2495b2dfaf9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="7bdf782f-2886-4011-99ee-a2495b2dfaf9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1596,14 +1637,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24B1C2B3-91A9-494D-BEB6-2B1BB33BE342}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{847D81C1-0646-4BD0-BC63-D9DF50568213}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="7bdf782f-2886-4011-99ee-a2495b2dfaf9"/>
@@ -1617,4 +1650,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24B1C2B3-91A9-494D-BEB6-2B1BB33BE342}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>